<commit_message>
Reduce to bare webserver for AWS ECS test
</commit_message>
<xml_diff>
--- a/deploy/aws price comparison 2023-05.xlsx
+++ b/deploy/aws price comparison 2023-05.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26626"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Attack_Vector\_attack_vector2\deploy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44685DFD-F3A5-40DD-A22A-8F839560C37D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08413259-B08E-48B2-A4D7-E484B8873DDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25395" yWindow="3075" windowWidth="21210" windowHeight="11475" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4260" yWindow="2730" windowWidth="37560" windowHeight="15885" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Application stats" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="41">
   <si>
     <t>Apprunner</t>
   </si>
@@ -144,6 +144,12 @@
   </si>
   <si>
     <t>year</t>
+  </si>
+  <si>
+    <t>AWS Nat gateway</t>
+  </si>
+  <si>
+    <t>per hour</t>
   </si>
 </sst>
 </file>
@@ -212,14 +218,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
@@ -722,18 +726,19 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60280056-7D27-4DE8-9E70-1BF0ACCE2D58}">
-  <dimension ref="A2:C27"/>
+  <dimension ref="A2:I27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
@@ -743,8 +748,17 @@
       <c r="C4" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="G4" t="s">
+        <v>39</v>
+      </c>
+      <c r="H4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>13</v>
       </c>
@@ -754,7 +768,7 @@
       </c>
       <c r="C5" s="4"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>15</v>
       </c>
@@ -766,7 +780,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -778,7 +792,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>37</v>
       </c>
@@ -790,7 +804,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>38</v>
       </c>
@@ -802,7 +816,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -813,7 +827,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
@@ -824,8 +838,8 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>19</v>
       </c>
       <c r="B13">
@@ -833,8 +847,8 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
         <v>20</v>
       </c>
       <c r="B14" s="3">
@@ -842,8 +856,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>21</v>
       </c>
       <c r="B15">
@@ -854,8 +868,8 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>22</v>
       </c>
       <c r="B16">
@@ -867,7 +881,7 @@
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="3" t="s">
         <v>23</v>
       </c>
       <c r="B17" s="3">

</xml_diff>